<commit_message>
random forest - experiment 2 multi-scale features
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="100900" yWindow="-5660" windowWidth="30300" windowHeight="21960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="103920" yWindow="-5660" windowWidth="27280" windowHeight="21660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -66,23 +66,23 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -481,10 +481,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="21.5" customWidth="1" style="3" min="1" max="11"/>
+    <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="23" customHeight="1">
@@ -545,43 +545,43 @@
       </c>
     </row>
     <row r="2" ht="85" customHeight="1">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="3" t="n">
         <v>46129</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>RandomForest</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>n_estimators=80, max_depth=20, class_weight=balanced_subscample, pixels_per_image=4000</t>
         </is>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="5" t="n">
         <v>0.926</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="4" t="n">
         <v>0.8869</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" s="4" t="n">
         <v>0.9024</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H2" s="4" t="n">
         <v>0.8313</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="6" t="n">
         <v>25.23</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J2" s="4" t="n">
         <v>6.5893</v>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>reproduction of Chris' baseline, 17 colour features.</t>
         </is>
@@ -1394,6 +1394,96 @@
       <c r="K20" t="inlineStr">
         <is>
           <t>val split, oob=0.9177</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-17 17:40:07</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>multiscale_sigma1248_3ch</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+12multiscale(a_lab,ExG,NGRDI @ sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.9474</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.9227</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.9331</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.8798</v>
+      </c>
+      <c r="I21" t="n">
+        <v>141.33</v>
+      </c>
+      <c r="J21" t="n">
+        <v>11.13</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>val split; oob=0.9456; experiment 2 — multi-scale features</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-19 11:20:20</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>multiscale_sigma1248_3ch</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+12multiscale(a_lab,ExG,NGRDI @ sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>0.9474</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.9227</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0.9331</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.8798</v>
+      </c>
+      <c r="I22" t="n">
+        <v>262.25</v>
+      </c>
+      <c r="J22" t="n">
+        <v>39.62</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>val split; oob=0.9456; experiment 2 — multi-scale features</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
random forest - experiment 3 feature ablation and importance
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1487,6 +1487,141 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-04-19 12:07:13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ablation_multiscale_a_lab_only</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+4multiscale(a_lab@sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>0.9509</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.9175</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.9321</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.8782</v>
+      </c>
+      <c r="I23" t="n">
+        <v>122.91</v>
+      </c>
+      <c r="J23" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>val split; oob=0.9413; ablation - multi-scale a_lab only</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-19 12:09:22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ablation_multiscale_exg_only</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+4multiscale(exg@sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>0.9474</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.9159</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.9294</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.8739</v>
+      </c>
+      <c r="I24" t="n">
+        <v>113.03</v>
+      </c>
+      <c r="J24" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>val split; oob=0.9422; ablation - multi-scale exg only</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-04-19 12:11:30</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ablation_multiscale_ngrdi_only</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+4multiscale(ngrdi@sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>0.9456</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.9102</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.9254</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.8673999999999999</v>
+      </c>
+      <c r="I25" t="n">
+        <v>111.69</v>
+      </c>
+      <c r="J25" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>val split; oob=0.9375; ablation - multi-scale ngrdi only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
random forest - final test eval
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1622,6 +1622,51 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-04-19 12:53:00</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>final_test_multiscale</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RandomForest</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>n_estimators=200, max_depth=20, min_samples_leaf=1, class_weight=balanced_subsample, features=17colour+12multiscale(a_lab,ExG,NGRDI@sigma=1,2,4,8)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>0.9457</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.9216</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.9321</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.8764</v>
+      </c>
+      <c r="I26" t="n">
+        <v>262.25</v>
+      </c>
+      <c r="J26" t="n">
+        <v>12.29</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>test split (FINAL) - rf_v2 multi-scale, one-shot evaluation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
knn - experiment 1 k sweep
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1667,6 +1667,231 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-04-19 16:32:49</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sweep_k3</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>n_neighbors=3, weights=uniform, algorithm=auto</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>0.9394</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.8931</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.9134</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.8499</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J27" t="n">
+        <v>154.89</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-04-19 16:35:42</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>sweep_k5</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>n_neighbors=5, weights=uniform, algorithm=auto</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0.9464</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.8917</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0.915</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.8532999999999999</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>172.99</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-04-19 16:38:31</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>sweep_k7</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>n_neighbors=7, weights=uniform, algorithm=auto</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>0.9509</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.8895</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0.9149</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.8538</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>168.9</v>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-04-19 16:41:25</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>sweep_k15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>n_neighbors=15, weights=uniform, algorithm=auto</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>0.9563</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.8833</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0.9116</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.8512</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>173.7</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-04-19 16:44:29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>sweep_k31</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>n_neighbors=31, weights=uniform, algorithm=auto</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>0.9584</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.8756</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0.9054</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.8451</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>183.54</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
knn - experiment 2 feature set comparison
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1892,6 +1892,51 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-04-19 18:39:16</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>feat_compare_17feat_k7</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>n_neighbors=7, weights=uniform, algorithm=auto, features=17colour, pixels_per_image=350</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.9045</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.9211</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.9103</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.8446</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J32" t="n">
+        <v>128.85</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels; compare to sweep_k7 (29 features)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
knn - experiment 3 weights sweep (uniform vs distance)
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1937,6 +1937,51 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-04-19 19:07:48</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>weights_distance_k7</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>n_neighbors=7, weights=distance, algorithm=auto, features=17colour+12multiscale(a_lab,ExG,NGRDI@sigma=1,2,4,8), pixels_per_image=350</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.9505</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.8895999999999999</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.9149</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.8537</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J33" t="n">
+        <v>135.92</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>val split; ~50k training pixels; compare to sweep_k7 (uniform weights)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
knn - final test eval
</commit_message>
<xml_diff>
--- a/ml/bm/training_results_history.xlsx
+++ b/ml/bm/training_results_history.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="21.5" customWidth="1" style="2" min="1" max="11"/>
@@ -1982,6 +1982,51 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-04-19 19:17:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>final_test_knn_k7</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>kNN</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>n_neighbors=7, weights=uniform, algorithm=auto, features=17colour+12multiscale(a_lab,ExG,NGRDI@sigma=1,2,4,8), pixels_per_image=350</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.9474</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.8967000000000001</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.9195</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.8578</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="J34" t="n">
+        <v>178.97</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>test split (FINAL) - kNN k=7 uniform, 29 features, one-shot evaluation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>